<commit_message>
Added pages, tests and E2E test file as well
</commit_message>
<xml_diff>
--- a/test-data/LoginData.xlsx
+++ b/test-data/LoginData.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="12">
   <si>
     <t>username</t>
   </si>
@@ -53,6 +53,9 @@
   </si>
   <si>
     <t>yes</t>
+  </si>
+  <si>
+    <t>no</t>
   </si>
 </sst>
 </file>
@@ -453,7 +456,7 @@
         <v>5</v>
       </c>
       <c r="D4" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
   </sheetData>

</xml_diff>